<commit_message>
Site guncellemesi - 17.09.2026 18:46
</commit_message>
<xml_diff>
--- a/app/borsa/gosterge-taramalari/data/düsüs-trendi.xlsx
+++ b/app/borsa/gosterge-taramalari/data/düsüs-trendi.xlsx
@@ -38,1861 +38,1861 @@
     <x:t>AFYON</x:t>
   </x:si>
   <x:si>
+    <x:t>AKFGY</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ALCTL</x:t>
+  </x:si>
+  <x:si>
     <x:t>ALGYO</x:t>
   </x:si>
   <x:si>
     <x:t>ARFYE</x:t>
   </x:si>
   <x:si>
+    <x:t>ATLAS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BRKVY</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BTCIM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BULGS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BURCE</x:t>
+  </x:si>
+  <x:si>
+    <x:t>CGCAM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>CIMSA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>CUSAN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DITAS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DMSAS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DOAS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ECILC</x:t>
+  </x:si>
+  <x:si>
+    <x:t>EGEGY</x:t>
+  </x:si>
+  <x:si>
+    <x:t>EKSUN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>EUYO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>FRIGO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>FRMPL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GARFA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GATEG</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GEDZA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GLRMK</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GRNYO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GRSEL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GSDHO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>HOROZ</x:t>
+  </x:si>
+  <x:si>
+    <x:t>IDGYO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>IHAAS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ISKPL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>IZENR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KAPLM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KIMMR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KRSTL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>LIDFA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>LILAK</x:t>
+  </x:si>
+  <x:si>
+    <x:t>LYDHO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MAALT</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MAGEN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MEGMT</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MEYSU</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MSGYO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MTRYO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ONCSM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>OYAYO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>OZKGY</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PAHOL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PENGD</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PINSU</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PNLSN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>QNBFK</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SEKFK</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SKBNK</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SKYLP</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SOKE</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TCELL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TTKOM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>UCAYM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>VAKFA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>VKGYO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>YUNSA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ZERGY</x:t>
+  </x:si>
+  <x:si>
+    <x:t>A1CAP</x:t>
+  </x:si>
+  <x:si>
+    <x:t>AAGYO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ACSEL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ADEL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ADESE</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ADGYO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>AEFES</x:t>
+  </x:si>
+  <x:si>
+    <x:t>AGESA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>AGHOL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>AGROT</x:t>
+  </x:si>
+  <x:si>
+    <x:t>AGYO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>AHGAZ</x:t>
+  </x:si>
+  <x:si>
+    <x:t>AHSGY</x:t>
+  </x:si>
+  <x:si>
+    <x:t>AKBNK</x:t>
+  </x:si>
+  <x:si>
+    <x:t>AKCNS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>AKENR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>AKFIS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>AKFYE</x:t>
+  </x:si>
+  <x:si>
+    <x:t>AKGRT</x:t>
+  </x:si>
+  <x:si>
+    <x:t>AKHAN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>AKMGY</x:t>
+  </x:si>
+  <x:si>
+    <x:t>AKSA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>AKSEN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>AKSGY</x:t>
+  </x:si>
+  <x:si>
+    <x:t>AKSUE</x:t>
+  </x:si>
+  <x:si>
+    <x:t>AKYHO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ALARK</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ALBRK</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ALBTN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ALCAR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ALFAS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ALKA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ALKIM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ALKLC</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ALTNY</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ALVES</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ANELE</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ANGEN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ANHYT</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ANSGR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ARASE</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ARCLK</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ARDYZ</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ARENA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ARMGD</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ARSAN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ARTMS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ARZUM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ASELS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ASGYO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ASTOR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ASUZU</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ATAGY</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ATAKP</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ATATP</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ATATR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ATEKS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ATSYH</x:t>
+  </x:si>
+  <x:si>
+    <x:t>AVGYO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>AVHOL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>AVOD</x:t>
+  </x:si>
+  <x:si>
+    <x:t>AVPGY</x:t>
+  </x:si>
+  <x:si>
+    <x:t>AVTUR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>AYCES</x:t>
+  </x:si>
+  <x:si>
+    <x:t>AYDEM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>AYEN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>AYES</x:t>
+  </x:si>
+  <x:si>
+    <x:t>AYGAZ</x:t>
+  </x:si>
+  <x:si>
+    <x:t>AZTEK</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BAGFS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BAHKM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BAKAB</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BALAT</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BALSU</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BANVT</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BARMA</x:t>
+  </x:si>
+  <x:si>
     <x:t>BASCM</x:t>
   </x:si>
   <x:si>
-    <x:t>BRKVY</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BTCIM</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BULGS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BURCE</x:t>
-  </x:si>
-  <x:si>
-    <x:t>CGCAM</x:t>
-  </x:si>
-  <x:si>
-    <x:t>CIMSA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>CUSAN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DITAS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DMSAS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DOAS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ECILC</x:t>
-  </x:si>
-  <x:si>
-    <x:t>EUYO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>FRIGO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>FRMPL</x:t>
+    <x:t>BASGZ</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BAYRK</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BEGYO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BERA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BESLR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BESTE</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BETAE</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BEYAZ</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BFREN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BIENY</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BIGCH</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BIGEN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BIGTK</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BIMAS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BINBN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BINHO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BIOEN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BIZIM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BJKAS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BLCYT</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BLUME</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BMSCH</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BMSTL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BNTAS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BOBET</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BORLS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BORSK</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BOSSA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BRISA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BRKO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BRKSN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BRLSM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BRMEN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BRSAN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BRYAT</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BSOKE</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BUCIM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BURVA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BVSAN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BYDNR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>CANTE</x:t>
+  </x:si>
+  <x:si>
+    <x:t>CASA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>CATES</x:t>
+  </x:si>
+  <x:si>
+    <x:t>CCOLA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>CELHA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>CEMAS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>CEMTS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>CEMZY</x:t>
+  </x:si>
+  <x:si>
+    <x:t>CEOEM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>CITAS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>CLEBI</x:t>
+  </x:si>
+  <x:si>
+    <x:t>CMBTN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>CMENT</x:t>
+  </x:si>
+  <x:si>
+    <x:t>CONSE</x:t>
+  </x:si>
+  <x:si>
+    <x:t>COSMO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>CRDFA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>CRFSA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>CVKMD</x:t>
+  </x:si>
+  <x:si>
+    <x:t>CWENE</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DAGI</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DAPGM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DARDL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DCTTR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DENGE</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DERHL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DERIM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DESA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DESPC</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DEVA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DGATE</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DGGYO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DGNMO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DIRIT</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DMRGD</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DNISI</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DOCO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DOFER</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DOFRB</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DOGUB</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DOHOL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DOKTA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DSTKF</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DUNYH</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DURDO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DURKN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DYOBY</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DZGYO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>EBEBK</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ECOGR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ECZYT</x:t>
+  </x:si>
+  <x:si>
+    <x:t>EDATA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>EDIP</x:t>
+  </x:si>
+  <x:si>
+    <x:t>EFOR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>EGEEN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>EGEPO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>EGGUB</x:t>
+  </x:si>
+  <x:si>
+    <x:t>EGPRO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>EGSER</x:t>
+  </x:si>
+  <x:si>
+    <x:t>EKDMR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>EKGYO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>EKIM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>EKIZ</x:t>
+  </x:si>
+  <x:si>
+    <x:t>EKOS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ELITE</x:t>
+  </x:si>
+  <x:si>
+    <x:t>EMKEL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>EMNIS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>EMPAE</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ENDAE</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ENERY</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ENJSA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ENKAI</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ENPRA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ENSRI</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ENTRA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>EPLAS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ERBOS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ERCB</x:t>
+  </x:si>
+  <x:si>
+    <x:t>EREGL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ERSU</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ESCAR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ESCOM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ESEN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ETILR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ETYAT</x:t>
+  </x:si>
+  <x:si>
+    <x:t>EUHOL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>EUKYO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>EUPWR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>EUREN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>EYGYO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>FADE</x:t>
+  </x:si>
+  <x:si>
+    <x:t>FENER</x:t>
+  </x:si>
+  <x:si>
+    <x:t>FLAP</x:t>
+  </x:si>
+  <x:si>
+    <x:t>FMIZP</x:t>
+  </x:si>
+  <x:si>
+    <x:t>FONET</x:t>
+  </x:si>
+  <x:si>
+    <x:t>FORMT</x:t>
+  </x:si>
+  <x:si>
+    <x:t>FORTE</x:t>
+  </x:si>
+  <x:si>
+    <x:t>FROTO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>FZLGY</x:t>
   </x:si>
   <x:si>
     <x:t>GARAN</x:t>
   </x:si>
   <x:si>
-    <x:t>GARFA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GEDZA</x:t>
+    <x:t>GEDIK</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GENIL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GENKM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GENTS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GEREL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GESAN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GIPTA</x:t>
   </x:si>
   <x:si>
     <x:t>GLBMD</x:t>
   </x:si>
   <x:si>
-    <x:t>GLRMK</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GRNYO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GRSEL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>HOROZ</x:t>
-  </x:si>
-  <x:si>
-    <x:t>IDGYO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>IHAAS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ISKPL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>IZENR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KAPLM</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KIMMR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KRSTL</x:t>
+    <x:t>GLCVY</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GLRYH</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GLYHO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GMTAS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GOKNR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GOLDA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GOLTS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GOODY</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GOZDE</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GRTHO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GSDDE</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GSRAY</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GUBRF</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GUNDG</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GWIND</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GZNMI</x:t>
+  </x:si>
+  <x:si>
+    <x:t>HALKB</x:t>
+  </x:si>
+  <x:si>
+    <x:t>HATEK</x:t>
+  </x:si>
+  <x:si>
+    <x:t>HATSN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>HDFGS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>HEDEF</x:t>
+  </x:si>
+  <x:si>
+    <x:t>HEKTS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>HKTM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>HLGYO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>HRKET</x:t>
+  </x:si>
+  <x:si>
+    <x:t>HTTBT</x:t>
+  </x:si>
+  <x:si>
+    <x:t>HUBVC</x:t>
+  </x:si>
+  <x:si>
+    <x:t>HUNER</x:t>
+  </x:si>
+  <x:si>
+    <x:t>HURGZ</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ICBCT</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ICUGS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>IEYHO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>IHEVA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>IHGZT</x:t>
+  </x:si>
+  <x:si>
+    <x:t>IHLAS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>IHLGM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>IHYAY</x:t>
+  </x:si>
+  <x:si>
+    <x:t>IMASM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>INDES</x:t>
+  </x:si>
+  <x:si>
+    <x:t>INFO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>INGRM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>INTEK</x:t>
+  </x:si>
+  <x:si>
+    <x:t>INTEM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>INVEO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>INVES</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ISATR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ISBIR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ISBTR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ISCTR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ISDMR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ISFIN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ISGSY</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ISGYO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ISKUR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ISMEN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ISSEN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ISVEA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ISYAT</x:t>
+  </x:si>
+  <x:si>
+    <x:t>IZFAS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>IZINV</x:t>
+  </x:si>
+  <x:si>
+    <x:t>IZMDC</x:t>
+  </x:si>
+  <x:si>
+    <x:t>JANTS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KARCL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KAREL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KARSN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KARTN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KATMR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KAYSE</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KBORU</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KCAER</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KCHOL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KENT</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KERVN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KFEIN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KGYO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KLGYO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KLKIM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KLMSN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KLNMA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KLRHO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KLSER</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KLSYN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KLYPV</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KMPUR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KNFRT</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KOCMT</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KONKA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KONTR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KONYA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KOPOL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KORDS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KOTON</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KPEKS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KRDMA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KRDMB</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KRDMD</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KRGYO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KRONT</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KRPLS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KRTEK</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KRVGD</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KSTUR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KTLEV</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KTSKR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KUTPO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KUVVA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KUYAS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KZBGY</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KZGYO</x:t>
   </x:si>
   <x:si>
     <x:t>LIDER</x:t>
   </x:si>
   <x:si>
-    <x:t>LIDFA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>LILAK</x:t>
-  </x:si>
-  <x:si>
-    <x:t>LYDHO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MAALT</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MAGEN</x:t>
+    <x:t>LINK</x:t>
+  </x:si>
+  <x:si>
+    <x:t>LKMNH</x:t>
+  </x:si>
+  <x:si>
+    <x:t>LMKDC</x:t>
+  </x:si>
+  <x:si>
+    <x:t>LOGO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>LRSHO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>LUKSK</x:t>
+  </x:si>
+  <x:si>
+    <x:t>LXGYO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>LYDYE</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MACKO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MAKIM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MAKTK</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MANAS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MARBL</x:t>
   </x:si>
   <x:si>
     <x:t>MARMR</x:t>
   </x:si>
   <x:si>
-    <x:t>MEGMT</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MEYSU</x:t>
+    <x:t>MARTI</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MASFN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MAVI</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MCARD</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MEDTR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MEGAP</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MEKAG</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MEPET</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MERCN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MERIT</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MERKO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>METEN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>METRO</x:t>
   </x:si>
   <x:si>
     <x:t>MGROS</x:t>
   </x:si>
   <x:si>
-    <x:t>MSGYO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MTRYO</x:t>
+    <x:t>MHRGY</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MIATK</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MMCAS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MNDRS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MNDTR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MOBTL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MOGAN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MOPAS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MPARK</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MRGYO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MRSHL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MTRKS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MZHLD</x:t>
+  </x:si>
+  <x:si>
+    <x:t>NATEN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>NETAS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>NETCD</x:t>
+  </x:si>
+  <x:si>
+    <x:t>NIBAS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>NTGAZ</x:t>
+  </x:si>
+  <x:si>
+    <x:t>NTHOL</x:t>
   </x:si>
   <x:si>
     <x:t>NUGYO</x:t>
   </x:si>
   <x:si>
-    <x:t>ONCSM</x:t>
-  </x:si>
-  <x:si>
-    <x:t>OYAYO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>OZKGY</x:t>
-  </x:si>
-  <x:si>
-    <x:t>PAHOL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>PENGD</x:t>
-  </x:si>
-  <x:si>
-    <x:t>PINSU</x:t>
-  </x:si>
-  <x:si>
-    <x:t>PNLSN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>QNBFK</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SEKFK</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SKBNK</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SKYLP</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SOKE</x:t>
+    <x:t>NUHCM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>OBAMS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>OBASE</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ODAS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ODINE</x:t>
+  </x:si>
+  <x:si>
+    <x:t>OFSYM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ONRYT</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ORCAY</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ORGE</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ORMA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ORZAX</x:t>
+  </x:si>
+  <x:si>
+    <x:t>OSMEN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>OSTIM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>OTKAR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>OTTO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>OYAKC</x:t>
+  </x:si>
+  <x:si>
+    <x:t>OYLUM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>OYYAT</x:t>
+  </x:si>
+  <x:si>
+    <x:t>OZATD</x:t>
+  </x:si>
+  <x:si>
+    <x:t>OZGYO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>OZRDN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>OZSUB</x:t>
+  </x:si>
+  <x:si>
+    <x:t>OZYSR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PAGYO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PAMEL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PAPIL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PARSN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PASEU</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PATEK</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PCILT</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PEKGY</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PENTA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PETKM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PETUN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PGSUS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PKART</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PKENT</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PLTUR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PNSUT</x:t>
+  </x:si>
+  <x:si>
+    <x:t>POLHO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>POLTK</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PRDGS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PRKAB</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PRKME</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PRZMA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PSDTC</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PSGYO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>QNBTR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>QUAGR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>QUICK</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RALYH</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RAYSG</x:t>
+  </x:si>
+  <x:si>
+    <x:t>REEDR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RGYAS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RNPOL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RODRG</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RTALB</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RUBNS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RUZYE</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RYGYO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RYSAS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SAFKR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SAHOL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SAMAT</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SANEL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SANFM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SANKO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SARAE</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SARKY</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SASA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SAYAS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SDTTR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SEGMN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SEGYO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SEKUR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SELEC</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SELVA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SERNT</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SEYKM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SILVR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SISE</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SKTAS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SKYMD</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SMART</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SMRTG</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SMRVA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SNGYO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SNICA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SNPAM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SODSN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SOHOE</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SOKM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SONME</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SRVGY</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SSAAT</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SUMAS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SUNTK</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SURGY</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SUWEN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SVGYO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TABGD</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TARKM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TATEN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TATGD</x:t>
   </x:si>
   <x:si>
     <x:t>TAVHL</x:t>
   </x:si>
   <x:si>
-    <x:t>TCELL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>UCAYM</x:t>
-  </x:si>
-  <x:si>
-    <x:t>VAKFA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>VKGYO</x:t>
+    <x:t>TBORG</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TCKRC</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TDGYO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TEHOL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TEKTU</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TERA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TEZOL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TGSAS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>THYAO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TKFEN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TKNKA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TKNSA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TLMAN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TMPOL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TMSN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TNZTP</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TOASO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TRALT</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TRCAS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TRENJ</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TRGYO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TRHOL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TRILC</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TRMET</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TSGYO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TSKB</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TSPOR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TTRAK</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TUCLK</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TUKAS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TUPRS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TUREX</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TURGG</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TURSG</x:t>
+  </x:si>
+  <x:si>
+    <x:t>UFUK</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ULAS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ULKER</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ULUFA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ULUSE</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ULUUN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>UMPAS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>UNLU</x:t>
+  </x:si>
+  <x:si>
+    <x:t>USAK</x:t>
+  </x:si>
+  <x:si>
+    <x:t>VAKBN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>VAKFN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>VAKKO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>VANGD</x:t>
+  </x:si>
+  <x:si>
+    <x:t>VBTYZ</x:t>
+  </x:si>
+  <x:si>
+    <x:t>VERTU</x:t>
+  </x:si>
+  <x:si>
+    <x:t>VERUS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>VESBE</x:t>
+  </x:si>
+  <x:si>
+    <x:t>VESTL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>VEYAS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>VKFYO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>VKING</x:t>
+  </x:si>
+  <x:si>
+    <x:t>VRGYO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>VSNMD</x:t>
+  </x:si>
+  <x:si>
+    <x:t>YAPRK</x:t>
+  </x:si>
+  <x:si>
+    <x:t>YATAS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>YAYLA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>YBTAS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>YEOTK</x:t>
+  </x:si>
+  <x:si>
+    <x:t>YESIL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>YGGYO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>YIGIT</x:t>
   </x:si>
   <x:si>
     <x:t>YKBNK</x:t>
   </x:si>
   <x:si>
-    <x:t>ZERGY</x:t>
-  </x:si>
-  <x:si>
-    <x:t>A1CAP</x:t>
-  </x:si>
-  <x:si>
-    <x:t>AAGYO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ACSEL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ADEL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ADESE</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ADGYO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>AEFES</x:t>
-  </x:si>
-  <x:si>
-    <x:t>AGESA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>AGHOL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>AGROT</x:t>
-  </x:si>
-  <x:si>
-    <x:t>AGYO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>AHGAZ</x:t>
-  </x:si>
-  <x:si>
-    <x:t>AHSGY</x:t>
-  </x:si>
-  <x:si>
-    <x:t>AKBNK</x:t>
-  </x:si>
-  <x:si>
-    <x:t>AKCNS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>AKENR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>AKFGY</x:t>
-  </x:si>
-  <x:si>
-    <x:t>AKFIS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>AKFYE</x:t>
-  </x:si>
-  <x:si>
-    <x:t>AKGRT</x:t>
-  </x:si>
-  <x:si>
-    <x:t>AKHAN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>AKMGY</x:t>
-  </x:si>
-  <x:si>
-    <x:t>AKSA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>AKSEN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>AKSGY</x:t>
-  </x:si>
-  <x:si>
-    <x:t>AKSUE</x:t>
-  </x:si>
-  <x:si>
-    <x:t>AKYHO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ALARK</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ALBRK</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ALBTN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ALCAR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ALCTL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ALFAS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ALKA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ALKIM</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ALKLC</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ALTNY</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ALVES</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ANELE</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ANGEN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ANHYT</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ANSGR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ARASE</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ARCLK</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ARDYZ</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ARENA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ARMGD</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ARSAN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ARTMS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ARZUM</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ASELS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ASGYO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ASTOR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ASUZU</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ATAGY</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ATAKP</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ATATP</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ATATR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ATEKS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ATLAS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ATSYH</x:t>
-  </x:si>
-  <x:si>
-    <x:t>AVGYO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>AVHOL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>AVOD</x:t>
-  </x:si>
-  <x:si>
-    <x:t>AVPGY</x:t>
-  </x:si>
-  <x:si>
-    <x:t>AVTUR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>AYCES</x:t>
-  </x:si>
-  <x:si>
-    <x:t>AYDEM</x:t>
-  </x:si>
-  <x:si>
-    <x:t>AYEN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>AYES</x:t>
-  </x:si>
-  <x:si>
-    <x:t>AYGAZ</x:t>
-  </x:si>
-  <x:si>
-    <x:t>AZTEK</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BAGFS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BAHKM</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BAKAB</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BALAT</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BALSU</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BANVT</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BARMA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BASGZ</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BAYRK</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BEGYO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BERA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BESLR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BESTE</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BETAE</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BEYAZ</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BFREN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BIENY</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BIGCH</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BIGEN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BIGTK</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BIMAS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BINBN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BINHO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BIOEN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BIZIM</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BJKAS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BLCYT</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BLUME</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BMSCH</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BMSTL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BNTAS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BOBET</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BORLS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BORSK</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BOSSA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BRISA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BRKO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BRKSN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BRLSM</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BRMEN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BRSAN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BRYAT</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BSOKE</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BUCIM</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BURVA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BVSAN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BYDNR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>CANTE</x:t>
-  </x:si>
-  <x:si>
-    <x:t>CASA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>CATES</x:t>
-  </x:si>
-  <x:si>
-    <x:t>CCOLA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>CELHA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>CEMAS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>CEMTS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>CEMZY</x:t>
-  </x:si>
-  <x:si>
-    <x:t>CEOEM</x:t>
-  </x:si>
-  <x:si>
-    <x:t>CITAS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>CLEBI</x:t>
-  </x:si>
-  <x:si>
-    <x:t>CMBTN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>CMENT</x:t>
-  </x:si>
-  <x:si>
-    <x:t>CONSE</x:t>
-  </x:si>
-  <x:si>
-    <x:t>COSMO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>CRDFA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>CRFSA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>CVKMD</x:t>
-  </x:si>
-  <x:si>
-    <x:t>CWENE</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DAGI</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DAPGM</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DARDL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DCTTR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DENGE</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DERHL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DERIM</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DESA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DESPC</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DEVA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DGATE</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DGGYO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DGNMO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DIRIT</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DMRGD</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DNISI</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DOCO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DOFER</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DOFRB</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DOGUB</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DOHOL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DOKTA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DSTKF</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DUNYH</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DURDO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DURKN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DYOBY</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DZGYO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>EBEBK</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ECOGR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ECZYT</x:t>
-  </x:si>
-  <x:si>
-    <x:t>EDATA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>EDIP</x:t>
-  </x:si>
-  <x:si>
-    <x:t>EFOR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>EGEEN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>EGEGY</x:t>
-  </x:si>
-  <x:si>
-    <x:t>EGEPO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>EGGUB</x:t>
-  </x:si>
-  <x:si>
-    <x:t>EGPRO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>EGSER</x:t>
-  </x:si>
-  <x:si>
-    <x:t>EKDMR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>EKGYO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>EKIM</x:t>
-  </x:si>
-  <x:si>
-    <x:t>EKIZ</x:t>
-  </x:si>
-  <x:si>
-    <x:t>EKOS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>EKSUN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ELITE</x:t>
-  </x:si>
-  <x:si>
-    <x:t>EMKEL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>EMNIS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>EMPAE</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ENDAE</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ENERY</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ENJSA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ENKAI</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ENPRA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ENSRI</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ENTRA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>EPLAS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ERBOS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ERCB</x:t>
-  </x:si>
-  <x:si>
-    <x:t>EREGL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ERSU</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ESCAR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ESCOM</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ESEN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ETILR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ETYAT</x:t>
-  </x:si>
-  <x:si>
-    <x:t>EUHOL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>EUKYO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>EUPWR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>EUREN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>EYGYO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>FADE</x:t>
-  </x:si>
-  <x:si>
-    <x:t>FENER</x:t>
-  </x:si>
-  <x:si>
-    <x:t>FLAP</x:t>
-  </x:si>
-  <x:si>
-    <x:t>FMIZP</x:t>
-  </x:si>
-  <x:si>
-    <x:t>FONET</x:t>
-  </x:si>
-  <x:si>
-    <x:t>FORMT</x:t>
-  </x:si>
-  <x:si>
-    <x:t>FORTE</x:t>
-  </x:si>
-  <x:si>
-    <x:t>FROTO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>FZLGY</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GATEG</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GEDIK</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GENIL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GENKM</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GENTS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GEREL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GESAN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GIPTA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GLCVY</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GLRYH</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GLYHO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GMTAS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GOKNR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GOLDA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GOLTS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GOODY</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GOZDE</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GRTHO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GSDDE</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GSDHO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GSRAY</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GUBRF</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GUNDG</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GWIND</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GZNMI</x:t>
-  </x:si>
-  <x:si>
-    <x:t>HALKB</x:t>
-  </x:si>
-  <x:si>
-    <x:t>HATEK</x:t>
-  </x:si>
-  <x:si>
-    <x:t>HATSN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>HDFGS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>HEDEF</x:t>
-  </x:si>
-  <x:si>
-    <x:t>HEKTS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>HKTM</x:t>
-  </x:si>
-  <x:si>
-    <x:t>HLGYO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>HRKET</x:t>
-  </x:si>
-  <x:si>
-    <x:t>HTTBT</x:t>
-  </x:si>
-  <x:si>
-    <x:t>HUBVC</x:t>
-  </x:si>
-  <x:si>
-    <x:t>HUNER</x:t>
-  </x:si>
-  <x:si>
-    <x:t>HURGZ</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ICBCT</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ICUGS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>IEYHO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>IHEVA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>IHGZT</x:t>
-  </x:si>
-  <x:si>
-    <x:t>IHLAS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>IHLGM</x:t>
-  </x:si>
-  <x:si>
-    <x:t>IHYAY</x:t>
-  </x:si>
-  <x:si>
-    <x:t>IMASM</x:t>
-  </x:si>
-  <x:si>
-    <x:t>INDES</x:t>
-  </x:si>
-  <x:si>
-    <x:t>INFO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>INGRM</x:t>
-  </x:si>
-  <x:si>
-    <x:t>INTEK</x:t>
-  </x:si>
-  <x:si>
-    <x:t>INTEM</x:t>
-  </x:si>
-  <x:si>
-    <x:t>INVEO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>INVES</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ISATR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ISBIR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ISBTR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ISCTR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ISDMR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ISFIN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ISGSY</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ISGYO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ISKUR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ISMEN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ISSEN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ISVEA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ISYAT</x:t>
-  </x:si>
-  <x:si>
-    <x:t>IZFAS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>IZINV</x:t>
-  </x:si>
-  <x:si>
-    <x:t>IZMDC</x:t>
-  </x:si>
-  <x:si>
-    <x:t>JANTS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KARCL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KAREL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KARSN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KARTN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KATMR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KAYSE</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KBORU</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KCAER</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KCHOL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KENT</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KERVN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KFEIN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KGYO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KLGYO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KLKIM</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KLMSN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KLNMA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KLRHO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KLSER</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KLSYN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KLYPV</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KMPUR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KNFRT</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KOCMT</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KONKA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KONTR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KONYA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KOPOL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KORDS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KOTON</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KPEKS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KRDMA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KRDMB</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KRDMD</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KRGYO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KRONT</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KRPLS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KRTEK</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KRVGD</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KSTUR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KTLEV</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KTSKR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KUTPO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KUVVA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KUYAS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KZBGY</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KZGYO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>LINK</x:t>
-  </x:si>
-  <x:si>
-    <x:t>LKMNH</x:t>
-  </x:si>
-  <x:si>
-    <x:t>LMKDC</x:t>
-  </x:si>
-  <x:si>
-    <x:t>LOGO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>LRSHO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>LUKSK</x:t>
-  </x:si>
-  <x:si>
-    <x:t>LXGYO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>LYDYE</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MACKO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MAKIM</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MAKTK</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MANAS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MARBL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MARTI</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MASFN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MAVI</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MCARD</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MEDTR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MEGAP</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MEKAG</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MEPET</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MERCN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MERIT</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MERKO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>METEN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>METRO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MHRGY</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MIATK</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MMCAS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MNDRS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MNDTR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MOBTL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MOGAN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MOPAS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MPARK</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MRGYO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MRSHL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MTRKS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MZHLD</x:t>
-  </x:si>
-  <x:si>
-    <x:t>NATEN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>NETAS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>NETCD</x:t>
-  </x:si>
-  <x:si>
-    <x:t>NIBAS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>NTGAZ</x:t>
-  </x:si>
-  <x:si>
-    <x:t>NTHOL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>NUHCM</x:t>
-  </x:si>
-  <x:si>
-    <x:t>OBAMS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>OBASE</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ODAS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ODINE</x:t>
-  </x:si>
-  <x:si>
-    <x:t>OFSYM</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ONRYT</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ORCAY</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ORGE</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ORMA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ORZAX</x:t>
-  </x:si>
-  <x:si>
-    <x:t>OSMEN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>OSTIM</x:t>
-  </x:si>
-  <x:si>
-    <x:t>OTKAR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>OTTO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>OYAKC</x:t>
-  </x:si>
-  <x:si>
-    <x:t>OYLUM</x:t>
-  </x:si>
-  <x:si>
-    <x:t>OYYAT</x:t>
-  </x:si>
-  <x:si>
-    <x:t>OZATD</x:t>
-  </x:si>
-  <x:si>
-    <x:t>OZGYO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>OZRDN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>OZSUB</x:t>
-  </x:si>
-  <x:si>
-    <x:t>OZYSR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>PAGYO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>PAMEL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>PAPIL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>PARSN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>PASEU</x:t>
-  </x:si>
-  <x:si>
-    <x:t>PATEK</x:t>
-  </x:si>
-  <x:si>
-    <x:t>PCILT</x:t>
-  </x:si>
-  <x:si>
-    <x:t>PEKGY</x:t>
-  </x:si>
-  <x:si>
-    <x:t>PENTA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>PETKM</x:t>
-  </x:si>
-  <x:si>
-    <x:t>PETUN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>PGSUS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>PKART</x:t>
-  </x:si>
-  <x:si>
-    <x:t>PKENT</x:t>
-  </x:si>
-  <x:si>
-    <x:t>PLTUR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>PNSUT</x:t>
-  </x:si>
-  <x:si>
-    <x:t>POLHO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>POLTK</x:t>
-  </x:si>
-  <x:si>
-    <x:t>PRDGS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>PRKAB</x:t>
-  </x:si>
-  <x:si>
-    <x:t>PRKME</x:t>
-  </x:si>
-  <x:si>
-    <x:t>PRZMA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>PSDTC</x:t>
-  </x:si>
-  <x:si>
-    <x:t>PSGYO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>QNBTR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>QUAGR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>QUICK</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RALYH</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RAYSG</x:t>
-  </x:si>
-  <x:si>
-    <x:t>REEDR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RGYAS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RNPOL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RODRG</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RTALB</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RUBNS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RUZYE</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RYGYO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RYSAS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SAFKR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SAHOL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SAMAT</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SANEL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SANFM</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SANKO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SARAE</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SARKY</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SASA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SAYAS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SDTTR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SEGMN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SEGYO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SEKUR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SELEC</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SELVA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SERNT</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SEYKM</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SILVR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SISE</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SKTAS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SKYMD</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SMART</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SMRTG</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SMRVA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SNGYO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SNICA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SNPAM</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SODSN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SOHOE</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SOKM</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SONME</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SRVGY</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SSAAT</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SUMAS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SUNTK</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SURGY</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SUWEN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SVGYO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TABGD</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TARKM</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TATEN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TATGD</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TBORG</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TCKRC</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TDGYO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TEHOL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TEKTU</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TERA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TEZOL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TGSAS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>THYAO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TKFEN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TKNKA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TKNSA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TLMAN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TMPOL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TMSN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TNZTP</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TOASO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TRALT</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TRCAS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TRENJ</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TRGYO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TRHOL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TRILC</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TRMET</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TSGYO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TSKB</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TSPOR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TTKOM</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TTRAK</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TUCLK</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TUKAS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TUPRS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TUREX</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TURGG</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TURSG</x:t>
-  </x:si>
-  <x:si>
-    <x:t>UFUK</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ULAS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ULKER</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ULUFA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ULUSE</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ULUUN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>UMPAS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>UNLU</x:t>
-  </x:si>
-  <x:si>
-    <x:t>USAK</x:t>
-  </x:si>
-  <x:si>
-    <x:t>VAKBN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>VAKFN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>VAKKO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>VANGD</x:t>
-  </x:si>
-  <x:si>
-    <x:t>VBTYZ</x:t>
-  </x:si>
-  <x:si>
-    <x:t>VERTU</x:t>
-  </x:si>
-  <x:si>
-    <x:t>VERUS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>VESBE</x:t>
-  </x:si>
-  <x:si>
-    <x:t>VESTL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>VEYAS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>VKFYO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>VKING</x:t>
-  </x:si>
-  <x:si>
-    <x:t>VRGYO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>VSNMD</x:t>
-  </x:si>
-  <x:si>
-    <x:t>YAPRK</x:t>
-  </x:si>
-  <x:si>
-    <x:t>YATAS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>YAYLA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>YBTAS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>YEOTK</x:t>
-  </x:si>
-  <x:si>
-    <x:t>YESIL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>YGGYO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>YIGIT</x:t>
-  </x:si>
-  <x:si>
     <x:t>YKSLN</x:t>
   </x:si>
   <x:si>
     <x:t>YONGA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>YUNSA</x:t>
   </x:si>
   <x:si>
     <x:t>YYAPI</x:t>

</xml_diff>